<commit_message>
Mise à jour auto - 2026-08-21 19:49
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bourse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C432EA-27E2-4A59-9ADB-512FD41BA7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304BB556-A4B7-404E-8823-569BEE1DF702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{F0554941-820F-4636-9443-571F98099751}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="160">
   <si>
     <t>14/08/2026</t>
   </si>
@@ -1176,7 +1176,7 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1337,7 +1337,7 @@
     <xf numFmtId="16" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1350,18 +1350,18 @@
     <xf numFmtId="10" fontId="6" fillId="8" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1369,7 +1369,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1385,29 +1385,26 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1436,7 +1433,7 @@
     <xf numFmtId="10" fontId="6" fillId="8" borderId="39" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="8" fillId="8" borderId="40" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1457,14 +1454,412 @@
     <cellStyle name="Normal 4" xfId="3" xr:uid="{1392998E-B22D-467D-85CD-A138D4CE51BA}"/>
     <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="212">
+  <dxfs count="105">
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
         <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
-        <color indexed="12"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
       </font>
     </dxf>
     <dxf>
@@ -1591,1378 +1986,6 @@
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
       </font>
     </dxf>
     <dxf>
@@ -19426,8 +18449,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="112" t="s">
-        <v>0</v>
+      <c r="A1" s="1">
+        <v>46255</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>1</v>
@@ -19438,13 +18461,13 @@
       <c r="D1" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="E1" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="114" t="s">
+      <c r="F1" s="111" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="115" t="s">
+      <c r="G1" s="112" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="7" t="s">
@@ -19465,13 +18488,13 @@
       <c r="A2" s="96">
         <v>1</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="106" t="s">
+      <c r="D2" s="15" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="16">
@@ -19480,7 +18503,7 @@
       <c r="F2" s="77">
         <v>0.34799999999999998</v>
       </c>
-      <c r="G2" s="116">
+      <c r="G2" s="113">
         <v>0</v>
       </c>
       <c r="I2" s="20"/>
@@ -19496,13 +18519,13 @@
       <c r="A3" s="98">
         <v>2</v>
       </c>
-      <c r="B3" s="105" t="s">
+      <c r="B3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="106" t="s">
+      <c r="D3" s="15" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="16">
@@ -19511,7 +18534,7 @@
       <c r="F3" s="77">
         <v>14.42</v>
       </c>
-      <c r="G3" s="116">
+      <c r="G3" s="113">
         <v>0</v>
       </c>
       <c r="H3" s="8"/>
@@ -19525,13 +18548,13 @@
       <c r="A4" s="96">
         <v>3</v>
       </c>
-      <c r="B4" s="105" t="s">
+      <c r="B4" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="106" t="s">
+      <c r="D4" s="15" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="16">
@@ -19540,7 +18563,7 @@
       <c r="F4" s="77">
         <v>75.95</v>
       </c>
-      <c r="G4" s="116">
+      <c r="G4" s="113">
         <v>0</v>
       </c>
       <c r="H4" s="8"/>
@@ -19554,13 +18577,13 @@
       <c r="A5" s="98">
         <v>4</v>
       </c>
-      <c r="B5" s="105" t="s">
+      <c r="B5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="105" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="106" t="s">
+      <c r="D5" s="15" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="16">
@@ -19569,7 +18592,7 @@
       <c r="F5" s="77">
         <v>71.739999999999995</v>
       </c>
-      <c r="G5" s="116">
+      <c r="G5" s="113">
         <v>0</v>
       </c>
       <c r="H5" s="8"/>
@@ -19583,13 +18606,13 @@
       <c r="A6" s="96">
         <v>5</v>
       </c>
-      <c r="B6" s="105" t="s">
+      <c r="B6" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="105" t="s">
+      <c r="C6" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="106" t="s">
+      <c r="D6" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="16">
@@ -19598,7 +18621,7 @@
       <c r="F6" s="77">
         <v>29.24</v>
       </c>
-      <c r="G6" s="116">
+      <c r="G6" s="113">
         <v>0</v>
       </c>
       <c r="H6" s="8"/>
@@ -19612,13 +18635,13 @@
       <c r="A7" s="98">
         <v>6</v>
       </c>
-      <c r="B7" s="105" t="s">
+      <c r="B7" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="105" t="s">
+      <c r="C7" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="106" t="s">
+      <c r="D7" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="16">
@@ -19627,7 +18650,7 @@
       <c r="F7" s="77">
         <v>76.05</v>
       </c>
-      <c r="G7" s="116">
+      <c r="G7" s="113">
         <v>0</v>
       </c>
       <c r="H7" s="8"/>
@@ -19641,13 +18664,13 @@
       <c r="A8" s="96">
         <v>7</v>
       </c>
-      <c r="B8" s="105" t="s">
+      <c r="B8" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="105" t="s">
+      <c r="C8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="106" t="s">
+      <c r="D8" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E8" s="16">
@@ -19656,7 +18679,7 @@
       <c r="F8" s="77">
         <v>0.115</v>
       </c>
-      <c r="G8" s="116">
+      <c r="G8" s="113">
         <v>0</v>
       </c>
       <c r="H8" s="8"/>
@@ -19670,13 +18693,13 @@
       <c r="A9" s="98">
         <v>8</v>
       </c>
-      <c r="B9" s="105" t="s">
+      <c r="B9" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="105" t="s">
+      <c r="C9" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="106" t="s">
+      <c r="D9" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="16">
@@ -19685,7 +18708,7 @@
       <c r="F9" s="77">
         <v>15.5</v>
       </c>
-      <c r="G9" s="116">
+      <c r="G9" s="113">
         <v>0</v>
       </c>
       <c r="H9" s="8"/>
@@ -19699,13 +18722,13 @@
       <c r="A10" s="96">
         <v>9</v>
       </c>
-      <c r="B10" s="105" t="s">
+      <c r="B10" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="105" t="s">
+      <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="106" t="s">
+      <c r="D10" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="16">
@@ -19714,7 +18737,7 @@
       <c r="F10" s="77">
         <v>0.8</v>
       </c>
-      <c r="G10" s="116">
+      <c r="G10" s="113">
         <v>0</v>
       </c>
       <c r="H10" s="8"/>
@@ -19728,13 +18751,13 @@
       <c r="A11" s="98">
         <v>10</v>
       </c>
-      <c r="B11" s="105" t="s">
+      <c r="B11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="105" t="s">
+      <c r="C11" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="106" t="s">
+      <c r="D11" s="15" t="s">
         <v>29</v>
       </c>
       <c r="E11" s="16">
@@ -19743,7 +18766,7 @@
       <c r="F11" s="77">
         <v>163.19999999999999</v>
       </c>
-      <c r="G11" s="116">
+      <c r="G11" s="113">
         <v>0</v>
       </c>
       <c r="H11" s="8"/>
@@ -19758,8 +18781,8 @@
       <c r="B12" s="100"/>
       <c r="C12" s="101"/>
       <c r="D12" s="102"/>
-      <c r="E12" s="117"/>
-      <c r="F12" s="118" t="s">
+      <c r="E12" s="114"/>
+      <c r="F12" s="115" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="39">
@@ -19819,13 +18842,13 @@
       <c r="A16" s="96">
         <v>1</v>
       </c>
-      <c r="B16" s="105" t="s">
+      <c r="B16" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="105" t="s">
+      <c r="C16" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="106" t="s">
+      <c r="D16" s="15" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="36">
@@ -19844,13 +18867,13 @@
       <c r="A17" s="98">
         <v>2</v>
       </c>
-      <c r="B17" s="105" t="s">
+      <c r="B17" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="105" t="s">
+      <c r="C17" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="106" t="s">
+      <c r="D17" s="15" t="s">
         <v>37</v>
       </c>
       <c r="E17" s="36">
@@ -19869,13 +18892,13 @@
       <c r="A18" s="96">
         <v>3</v>
       </c>
-      <c r="B18" s="105" t="s">
+      <c r="B18" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="105" t="s">
+      <c r="C18" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D18" s="106" t="s">
+      <c r="D18" s="15" t="s">
         <v>39</v>
       </c>
       <c r="E18" s="36">
@@ -19894,13 +18917,13 @@
       <c r="A19" s="98">
         <v>4</v>
       </c>
-      <c r="B19" s="105" t="s">
+      <c r="B19" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="105" t="s">
+      <c r="C19" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="106" t="s">
+      <c r="D19" s="15" t="s">
         <v>41</v>
       </c>
       <c r="E19" s="36">
@@ -19919,13 +18942,13 @@
       <c r="A20" s="96">
         <v>5</v>
       </c>
-      <c r="B20" s="105" t="s">
+      <c r="B20" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="105" t="s">
+      <c r="C20" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="106" t="s">
+      <c r="D20" s="15" t="s">
         <v>43</v>
       </c>
       <c r="E20" s="36">
@@ -19944,13 +18967,13 @@
       <c r="A21" s="98">
         <v>6</v>
       </c>
-      <c r="B21" s="105" t="s">
+      <c r="B21" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="105" t="s">
+      <c r="C21" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="106" t="s">
+      <c r="D21" s="15" t="s">
         <v>45</v>
       </c>
       <c r="E21" s="36">
@@ -19969,13 +18992,13 @@
       <c r="A22" s="96">
         <v>7</v>
       </c>
-      <c r="B22" s="105" t="s">
+      <c r="B22" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="105" t="s">
+      <c r="C22" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="106" t="s">
+      <c r="D22" s="15" t="s">
         <v>47</v>
       </c>
       <c r="E22" s="36">
@@ -19994,13 +19017,13 @@
       <c r="A23" s="98">
         <v>8</v>
       </c>
-      <c r="B23" s="105" t="s">
+      <c r="B23" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="105" t="s">
+      <c r="C23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="106" t="s">
+      <c r="D23" s="15" t="s">
         <v>49</v>
       </c>
       <c r="E23" s="36">
@@ -20019,13 +19042,13 @@
       <c r="A24" s="96">
         <v>9</v>
       </c>
-      <c r="B24" s="105" t="s">
+      <c r="B24" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="105" t="s">
+      <c r="C24" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="106" t="s">
+      <c r="D24" s="15" t="s">
         <v>51</v>
       </c>
       <c r="E24" s="36">
@@ -20044,13 +19067,13 @@
       <c r="A25" s="98">
         <v>10</v>
       </c>
-      <c r="B25" s="105" t="s">
+      <c r="B25" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="105" t="s">
+      <c r="C25" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D25" s="106" t="s">
+      <c r="D25" s="15" t="s">
         <v>53</v>
       </c>
       <c r="E25" s="36">
@@ -20067,9 +19090,9 @@
     </row>
     <row r="26" spans="1:11" ht="15.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="96"/>
-      <c r="B26" s="105"/>
+      <c r="B26" s="14"/>
       <c r="C26" s="76"/>
-      <c r="D26" s="107"/>
+      <c r="D26" s="105"/>
       <c r="E26" s="36"/>
       <c r="F26" s="38" t="s">
         <v>30</v>
@@ -20091,11 +19114,11 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A27" s="108"/>
-      <c r="B27" s="109"/>
+      <c r="A27" s="106"/>
+      <c r="B27" s="107"/>
       <c r="C27" s="100"/>
-      <c r="D27" s="110"/>
-      <c r="E27" s="111"/>
+      <c r="D27" s="108"/>
+      <c r="E27" s="109"/>
       <c r="F27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27"/>
@@ -20117,13 +19140,13 @@
       <c r="D29" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="E29" s="113" t="s">
+      <c r="E29" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="F29" s="114" t="s">
+      <c r="F29" s="111" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="115" t="s">
+      <c r="G29" s="112" t="s">
         <v>6</v>
       </c>
       <c r="H29" s="7" t="s">
@@ -20135,13 +19158,13 @@
       <c r="A30" s="96">
         <v>1</v>
       </c>
-      <c r="B30" s="105" t="s">
+      <c r="B30" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="105" t="s">
+      <c r="C30" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D30" s="106" t="s">
+      <c r="D30" s="15" t="s">
         <v>57</v>
       </c>
       <c r="E30" s="16">
@@ -20150,7 +19173,7 @@
       <c r="F30" s="77">
         <v>11.4</v>
       </c>
-      <c r="G30" s="116">
+      <c r="G30" s="113">
         <v>0</v>
       </c>
       <c r="H30"/>
@@ -20160,13 +19183,13 @@
       <c r="A31" s="98">
         <v>2</v>
       </c>
-      <c r="B31" s="105" t="s">
+      <c r="B31" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C31" s="105" t="s">
+      <c r="C31" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D31" s="106" t="s">
+      <c r="D31" s="15" t="s">
         <v>59</v>
       </c>
       <c r="E31" s="16">
@@ -20175,7 +19198,7 @@
       <c r="F31" s="77">
         <v>21.75</v>
       </c>
-      <c r="G31" s="116">
+      <c r="G31" s="113">
         <v>0</v>
       </c>
       <c r="H31"/>
@@ -20185,13 +19208,13 @@
       <c r="A32" s="96">
         <v>3</v>
       </c>
-      <c r="B32" s="105" t="s">
+      <c r="B32" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="C32" s="105" t="s">
+      <c r="C32" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D32" s="106" t="s">
+      <c r="D32" s="15" t="s">
         <v>61</v>
       </c>
       <c r="E32" s="16">
@@ -20200,7 +19223,7 @@
       <c r="F32" s="77">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="G32" s="116">
+      <c r="G32" s="113">
         <v>0</v>
       </c>
       <c r="H32"/>
@@ -20210,13 +19233,13 @@
       <c r="A33" s="98">
         <v>4</v>
       </c>
-      <c r="B33" s="105" t="s">
+      <c r="B33" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="105" t="s">
+      <c r="C33" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D33" s="106" t="s">
+      <c r="D33" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E33" s="16">
@@ -20225,7 +19248,7 @@
       <c r="F33" s="77">
         <v>0.38</v>
       </c>
-      <c r="G33" s="116">
+      <c r="G33" s="113">
         <v>0</v>
       </c>
       <c r="H33"/>
@@ -20235,13 +19258,13 @@
       <c r="A34" s="96">
         <v>5</v>
       </c>
-      <c r="B34" s="105" t="s">
+      <c r="B34" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="105" t="s">
+      <c r="C34" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D34" s="106" t="s">
+      <c r="D34" s="15" t="s">
         <v>65</v>
       </c>
       <c r="E34" s="16">
@@ -20250,7 +19273,7 @@
       <c r="F34" s="77">
         <v>1.79</v>
       </c>
-      <c r="G34" s="116">
+      <c r="G34" s="113">
         <v>0</v>
       </c>
       <c r="H34"/>
@@ -20260,13 +19283,13 @@
       <c r="A35" s="98">
         <v>6</v>
       </c>
-      <c r="B35" s="105" t="s">
+      <c r="B35" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="105" t="s">
+      <c r="C35" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D35" s="106" t="s">
+      <c r="D35" s="15" t="s">
         <v>67</v>
       </c>
       <c r="E35" s="16">
@@ -20275,7 +19298,7 @@
       <c r="F35" s="77">
         <v>3</v>
       </c>
-      <c r="G35" s="116">
+      <c r="G35" s="113">
         <v>0</v>
       </c>
       <c r="H35"/>
@@ -20285,13 +19308,13 @@
       <c r="A36" s="96">
         <v>7</v>
       </c>
-      <c r="B36" s="105" t="s">
+      <c r="B36" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="105" t="s">
+      <c r="C36" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="106" t="s">
+      <c r="D36" s="15" t="s">
         <v>69</v>
       </c>
       <c r="E36" s="16">
@@ -20300,7 +19323,7 @@
       <c r="F36" s="77">
         <v>0.13600000000000001</v>
       </c>
-      <c r="G36" s="116">
+      <c r="G36" s="113">
         <v>0</v>
       </c>
       <c r="H36"/>
@@ -20310,13 +19333,13 @@
       <c r="A37" s="98">
         <v>8</v>
       </c>
-      <c r="B37" s="105" t="s">
+      <c r="B37" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="105" t="s">
+      <c r="C37" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D37" s="106" t="s">
+      <c r="D37" s="15" t="s">
         <v>72</v>
       </c>
       <c r="E37" s="16">
@@ -20325,7 +19348,7 @@
       <c r="F37" s="77">
         <v>3.19</v>
       </c>
-      <c r="G37" s="116">
+      <c r="G37" s="113">
         <v>0</v>
       </c>
       <c r="H37"/>
@@ -20336,13 +19359,13 @@
       <c r="A38" s="96">
         <v>9</v>
       </c>
-      <c r="B38" s="105" t="s">
+      <c r="B38" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="C38" s="105" t="s">
+      <c r="C38" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="106" t="s">
+      <c r="D38" s="15" t="s">
         <v>74</v>
       </c>
       <c r="E38" s="16">
@@ -20351,7 +19374,7 @@
       <c r="F38" s="77">
         <v>0.58799999999999997</v>
       </c>
-      <c r="G38" s="116">
+      <c r="G38" s="113">
         <v>0</v>
       </c>
       <c r="H38"/>
@@ -20362,13 +19385,13 @@
       <c r="A39" s="98">
         <v>10</v>
       </c>
-      <c r="B39" s="105" t="s">
+      <c r="B39" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C39" s="105" t="s">
+      <c r="C39" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D39" s="106" t="s">
+      <c r="D39" s="15" t="s">
         <v>76</v>
       </c>
       <c r="E39" s="16">
@@ -20377,22 +19400,22 @@
       <c r="F39" s="77">
         <v>0.158</v>
       </c>
-      <c r="G39" s="116">
+      <c r="G39" s="113">
         <v>0</v>
       </c>
       <c r="H39"/>
       <c r="I39"/>
     </row>
     <row r="40" spans="1:16" ht="15.9" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="125"/>
-      <c r="B40" s="126"/>
-      <c r="C40" s="127"/>
-      <c r="D40" s="128"/>
-      <c r="E40" s="129"/>
-      <c r="F40" s="118" t="s">
+      <c r="A40" s="122"/>
+      <c r="B40" s="123"/>
+      <c r="C40" s="124"/>
+      <c r="D40" s="125"/>
+      <c r="E40" s="126"/>
+      <c r="F40" s="115" t="s">
         <v>30</v>
       </c>
-      <c r="G40" s="130">
+      <c r="G40" s="127">
         <v>0</v>
       </c>
       <c r="H40">
@@ -20423,13 +19446,13 @@
       <c r="D42" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="E42" s="113" t="s">
+      <c r="E42" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="F42" s="114" t="s">
+      <c r="F42" s="111" t="s">
         <v>5</v>
       </c>
-      <c r="G42" s="121" t="s">
+      <c r="G42" s="118" t="s">
         <v>6</v>
       </c>
       <c r="H42" s="7" t="s">
@@ -20441,12 +19464,12 @@
       <c r="A43" s="96">
         <v>1</v>
       </c>
-      <c r="B43" s="105"/>
-      <c r="C43" s="105"/>
-      <c r="D43" s="106"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="15"/>
       <c r="E43" s="16"/>
       <c r="F43" s="77"/>
-      <c r="G43" s="122"/>
+      <c r="G43" s="119"/>
       <c r="H43"/>
       <c r="I43"/>
     </row>
@@ -20454,12 +19477,12 @@
       <c r="A44" s="98">
         <v>2</v>
       </c>
-      <c r="B44" s="105"/>
-      <c r="C44" s="105"/>
-      <c r="D44" s="106"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="15"/>
       <c r="E44" s="16"/>
       <c r="F44" s="77"/>
-      <c r="G44" s="122"/>
+      <c r="G44" s="119"/>
       <c r="H44"/>
       <c r="I44"/>
     </row>
@@ -20467,12 +19490,12 @@
       <c r="A45" s="96">
         <v>3</v>
       </c>
-      <c r="B45" s="105"/>
-      <c r="C45" s="105"/>
-      <c r="D45" s="106"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="15"/>
       <c r="E45" s="16"/>
       <c r="F45" s="77"/>
-      <c r="G45" s="122"/>
+      <c r="G45" s="119"/>
       <c r="H45"/>
       <c r="I45"/>
     </row>
@@ -20480,12 +19503,12 @@
       <c r="A46" s="98">
         <v>4</v>
       </c>
-      <c r="B46" s="105"/>
-      <c r="C46" s="105"/>
-      <c r="D46" s="106"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="15"/>
       <c r="E46" s="16"/>
       <c r="F46" s="77"/>
-      <c r="G46" s="122"/>
+      <c r="G46" s="119"/>
       <c r="H46"/>
       <c r="I46"/>
     </row>
@@ -20493,12 +19516,12 @@
       <c r="A47" s="96">
         <v>5</v>
       </c>
-      <c r="B47" s="105"/>
-      <c r="C47" s="105"/>
-      <c r="D47" s="106"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="15"/>
       <c r="E47" s="16"/>
       <c r="F47" s="77"/>
-      <c r="G47" s="122"/>
+      <c r="G47" s="119"/>
       <c r="H47"/>
       <c r="I47"/>
     </row>
@@ -20506,12 +19529,12 @@
       <c r="A48" s="98">
         <v>6</v>
       </c>
-      <c r="B48" s="105"/>
-      <c r="C48" s="105"/>
-      <c r="D48" s="106"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="15"/>
       <c r="E48" s="16"/>
       <c r="F48" s="77"/>
-      <c r="G48" s="122"/>
+      <c r="G48" s="119"/>
       <c r="H48"/>
       <c r="I48"/>
     </row>
@@ -20519,12 +19542,12 @@
       <c r="A49" s="96">
         <v>7</v>
       </c>
-      <c r="B49" s="105"/>
-      <c r="C49" s="105"/>
-      <c r="D49" s="106"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="15"/>
       <c r="E49" s="16"/>
       <c r="F49" s="77"/>
-      <c r="G49" s="122"/>
+      <c r="G49" s="119"/>
       <c r="H49"/>
       <c r="I49"/>
     </row>
@@ -20532,12 +19555,12 @@
       <c r="A50" s="98">
         <v>8</v>
       </c>
-      <c r="B50" s="105"/>
-      <c r="C50" s="105"/>
-      <c r="D50" s="106"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="15"/>
       <c r="E50" s="16"/>
       <c r="F50" s="77"/>
-      <c r="G50" s="122"/>
+      <c r="G50" s="119"/>
       <c r="H50"/>
       <c r="I50"/>
     </row>
@@ -20545,12 +19568,12 @@
       <c r="A51" s="96">
         <v>9</v>
       </c>
-      <c r="B51" s="105"/>
-      <c r="C51" s="105"/>
-      <c r="D51" s="106"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="15"/>
       <c r="E51" s="16"/>
       <c r="F51" s="77"/>
-      <c r="G51" s="122"/>
+      <c r="G51" s="119"/>
       <c r="H51"/>
       <c r="I51"/>
     </row>
@@ -20558,12 +19581,12 @@
       <c r="A52" s="98">
         <v>10</v>
       </c>
-      <c r="B52" s="105"/>
-      <c r="C52" s="105"/>
-      <c r="D52" s="106"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="15"/>
       <c r="E52" s="16"/>
       <c r="F52" s="77"/>
-      <c r="G52" s="122"/>
+      <c r="G52" s="119"/>
       <c r="H52"/>
       <c r="I52"/>
     </row>
@@ -20572,11 +19595,11 @@
       <c r="B53" s="100"/>
       <c r="C53" s="101"/>
       <c r="D53" s="102"/>
-      <c r="E53" s="123"/>
-      <c r="F53" s="120" t="s">
+      <c r="E53" s="120"/>
+      <c r="F53" s="117" t="s">
         <v>30</v>
       </c>
-      <c r="G53" s="124">
+      <c r="G53" s="121">
         <v>0</v>
       </c>
       <c r="H53" s="31" t="s">
@@ -21165,7 +20188,7 @@
         <v>4</v>
       </c>
       <c r="B85" s="80"/>
-      <c r="C85" s="119"/>
+      <c r="C85" s="116"/>
       <c r="D85" s="80"/>
       <c r="E85" s="16"/>
       <c r="F85" s="77"/>
@@ -21178,7 +20201,7 @@
         <v>5</v>
       </c>
       <c r="B86" s="75"/>
-      <c r="C86" s="119"/>
+      <c r="C86" s="116"/>
       <c r="D86" s="75"/>
       <c r="E86" s="16"/>
       <c r="F86" s="77"/>
@@ -21191,7 +20214,7 @@
         <v>6</v>
       </c>
       <c r="B87" s="80"/>
-      <c r="C87" s="119"/>
+      <c r="C87" s="116"/>
       <c r="D87" s="80"/>
       <c r="E87" s="16"/>
       <c r="F87" s="77"/>
@@ -21217,7 +20240,7 @@
         <v>8</v>
       </c>
       <c r="B89" s="80"/>
-      <c r="C89" s="119"/>
+      <c r="C89" s="116"/>
       <c r="D89" s="80"/>
       <c r="E89" s="16"/>
       <c r="F89" s="77"/>
@@ -21257,7 +20280,7 @@
       <c r="C92" s="83"/>
       <c r="D92" s="54"/>
       <c r="E92" s="84"/>
-      <c r="F92" s="120" t="s">
+      <c r="F92" s="117" t="s">
         <v>30</v>
       </c>
       <c r="G92" s="50" t="e">
@@ -23681,76 +22704,73 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B56:B65">
-    <cfRule type="expression" dxfId="105" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="104" priority="5" stopIfTrue="1">
       <formula>IF(AO56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:B78">
-    <cfRule type="expression" dxfId="104" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="103" priority="3" stopIfTrue="1">
       <formula>IF(AO69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B81">
-    <cfRule type="expression" dxfId="103" priority="50" stopIfTrue="1">
+    <cfRule type="expression" dxfId="102" priority="50" stopIfTrue="1">
       <formula>IF(AN62&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B82:B91">
-    <cfRule type="expression" dxfId="102" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="101" priority="9" stopIfTrue="1">
       <formula>IF(AL82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="expression" dxfId="101" priority="46" stopIfTrue="1">
+    <cfRule type="expression" dxfId="100" priority="46" stopIfTrue="1">
       <formula>IF(AL91&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="expression" dxfId="100" priority="49" stopIfTrue="1">
+    <cfRule type="expression" dxfId="99" priority="49" stopIfTrue="1">
       <formula>IF(AN75&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:B105">
-    <cfRule type="expression" dxfId="99" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="98" priority="7" stopIfTrue="1">
       <formula>IF(AO96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B106">
-    <cfRule type="expression" dxfId="98" priority="47" stopIfTrue="1">
+    <cfRule type="expression" dxfId="97" priority="47" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="expression" dxfId="97" priority="48" stopIfTrue="1">
+    <cfRule type="expression" dxfId="96" priority="48" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D56:D65">
-    <cfRule type="expression" dxfId="96" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="95" priority="4" stopIfTrue="1">
       <formula>IF(AQ56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:D78">
-    <cfRule type="expression" dxfId="95" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="94" priority="2" stopIfTrue="1">
       <formula>IF(AQ69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82:D91">
-    <cfRule type="expression" dxfId="94" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="93" priority="8" stopIfTrue="1">
       <formula>IF(AN82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D96:D105">
-    <cfRule type="expression" dxfId="93" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="92" priority="6" stopIfTrue="1">
       <formula>IF(AQ96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" dxfId="92" priority="19" stopIfTrue="1">
+    <cfRule type="expression" dxfId="91" priority="19" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="91" priority="20" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="90" priority="21" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
@@ -23764,33 +22784,33 @@
     <cfRule type="expression" dxfId="87" priority="24" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="86" priority="20" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" dxfId="86" priority="80" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="85" priority="85" stopIfTrue="1">
+      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="85" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="84" priority="84" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="84" priority="82" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="83" priority="83" stopIfTrue="1">
       <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="82" priority="84" stopIfTrue="1">
+    <cfRule type="expression" dxfId="82" priority="82" stopIfTrue="1">
+      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="81" priority="81" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="85" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="80" priority="80" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" dxfId="80" priority="86" stopIfTrue="1">
+    <cfRule type="expression" dxfId="79" priority="86" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="79" priority="87" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="78" priority="88" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
@@ -23804,306 +22824,308 @@
     <cfRule type="expression" dxfId="75" priority="91" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="74" priority="87" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F56">
-    <cfRule type="expression" dxfId="74" priority="76" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="73" priority="78" stopIfTrue="1">
+      <formula>IF($T254="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="72" priority="77" stopIfTrue="1">
       <formula>IF($AN28="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="72" priority="78" stopIfTrue="1">
-      <formula>IF($T254="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="71" priority="79" stopIfTrue="1">
       <formula>IF($U254="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" dxfId="70" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="F56:F67">
+    <cfRule type="expression" dxfId="70" priority="76" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F57:F67">
+    <cfRule type="expression" dxfId="69" priority="95" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="68" priority="93" stopIfTrue="1">
+      <formula>IF($AK29="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="67" priority="94" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69">
+    <cfRule type="expression" dxfId="66" priority="97" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="96" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="64" priority="98" stopIfTrue="1">
+      <formula>IF($AJ43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="63" priority="99" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="62" priority="100" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" dxfId="61" priority="1" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F70:F78">
+    <cfRule type="expression" dxfId="60" priority="103" stopIfTrue="1">
+      <formula>IF($U267="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="59" priority="102" stopIfTrue="1">
+      <formula>IF($T267="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="58" priority="101" stopIfTrue="1">
+      <formula>IF($AJ42="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" dxfId="57" priority="106" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="56" priority="104" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="55" priority="105" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" dxfId="69" priority="65" stopIfTrue="1">
+    <cfRule type="expression" dxfId="54" priority="65" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" dxfId="68" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="53" priority="68" stopIfTrue="1">
+      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="52" priority="66" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="51" priority="67" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="66" priority="68" stopIfTrue="1">
-      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" dxfId="65" priority="73" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="64" priority="74" stopIfTrue="1">
+    <cfRule type="expression" dxfId="50" priority="74" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="75" stopIfTrue="1">
+    <cfRule type="expression" dxfId="49" priority="75" stopIfTrue="1">
       <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="73" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" dxfId="62" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="47" priority="69" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" dxfId="61" priority="70" stopIfTrue="1">
+    <cfRule type="expression" dxfId="46" priority="70" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="71" stopIfTrue="1">
+    <cfRule type="expression" dxfId="45" priority="71" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="72" stopIfTrue="1">
+    <cfRule type="expression" dxfId="44" priority="72" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="58" priority="52" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
+    <cfRule type="cellIs" dxfId="43" priority="53" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="52" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="53" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12 G16:G28">
+    <cfRule type="cellIs" dxfId="41" priority="25" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:G41 G2:G12 G16:G26">
+    <cfRule type="cellIs" dxfId="40" priority="51" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G28 G2:G12">
-    <cfRule type="cellIs" dxfId="56" priority="25" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="55" priority="51" operator="greaterThan">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G54 G56:G67 G30:G41">
-    <cfRule type="cellIs" dxfId="54" priority="42" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G43:G54 G30:G41 G56:G67">
+    <cfRule type="cellIs" dxfId="39" priority="42" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" dxfId="53" priority="30" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="38" priority="30" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="31" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="37" priority="33" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="32" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="36" priority="32" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="33" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="35" priority="31" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" dxfId="49" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="34" priority="16" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="17" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="33" priority="18" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="17" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="18" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" dxfId="46" priority="43" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="45" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="44" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="43" operator="greaterThan">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="44" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="45" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" dxfId="43" priority="26" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="29" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="27" operator="greaterThan">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="26" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="27" operator="greaterThan">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="28" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="28" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="29" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" dxfId="39" priority="38" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="40" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="39" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="40" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="41" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="38" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="41" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" dxfId="35" priority="34" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="37" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="36" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="35" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="35" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="36" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="34" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="37" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H81">
+    <cfRule type="cellIs" dxfId="16" priority="15" operator="greaterThan">
+      <formula>$H81</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I12 I53 K53 I66 K66">
-    <cfRule type="cellIs" dxfId="31" priority="59" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="59" operator="greaterThan">
       <formula>$K12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26">
-    <cfRule type="cellIs" dxfId="30" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="greaterThan">
       <formula>$K26</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I75">
-    <cfRule type="cellIs" dxfId="29" priority="60" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="60" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I93:I94">
-    <cfRule type="cellIs" dxfId="28" priority="58" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="58" operator="greaterThan">
       <formula>$K93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I107">
-    <cfRule type="cellIs" dxfId="27" priority="57" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="57" operator="greaterThan">
       <formula>$K107</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I109">
-    <cfRule type="cellIs" dxfId="26" priority="55" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="55" operator="greaterThan">
       <formula>$K109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J97">
-    <cfRule type="cellIs" dxfId="25" priority="62" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="62" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J103">
-    <cfRule type="cellIs" dxfId="24" priority="61" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="61" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="cellIs" dxfId="23" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="13" operator="greaterThan">
       <formula>$K12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="cellIs" dxfId="22" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="12" operator="greaterThan">
       <formula>$K26</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K41">
-    <cfRule type="cellIs" dxfId="21" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="11" operator="greaterThan">
       <formula>$K41</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" dxfId="20" priority="15" operator="greaterThan">
-      <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="K93:K94">
-    <cfRule type="cellIs" dxfId="19" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="14" operator="greaterThan">
       <formula>$K93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K104">
-    <cfRule type="cellIs" dxfId="18" priority="63" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="63" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K107">
-    <cfRule type="cellIs" dxfId="17" priority="56" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="56" operator="greaterThan">
       <formula>$I107</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K109">
-    <cfRule type="cellIs" dxfId="16" priority="54" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="54" operator="greaterThan">
       <formula>$I109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P37:P38">
-    <cfRule type="cellIs" dxfId="15" priority="64" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="64" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F57:F67">
-    <cfRule type="expression" dxfId="14" priority="92" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="93" stopIfTrue="1">
-      <formula>IF($AK29="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="94" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="11" priority="95" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69">
-    <cfRule type="expression" dxfId="10" priority="96" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="97" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="98" stopIfTrue="1">
-      <formula>IF($AJ43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="99" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="100" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F70:F78">
-    <cfRule type="expression" dxfId="5" priority="101" stopIfTrue="1">
-      <formula>IF($AJ42="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="102" stopIfTrue="1">
-      <formula>IF($T267="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="103" stopIfTrue="1">
-      <formula>IF($U267="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" dxfId="2" priority="104" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="105" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="106" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Mise à jour auto - 2026-09-04 20:03
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bourse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F429416-0EC9-49A1-90B2-3FFF5941422E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE97C68-D717-401F-B5F4-13D0882D2076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{A7B67D64-2DDB-46B6-9CAD-5E62F326C346}"/>
   </bookViews>
@@ -1152,7 +1152,7 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1313,7 +1313,7 @@
     <xf numFmtId="16" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1326,18 +1326,18 @@
     <xf numFmtId="10" fontId="6" fillId="8" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1345,7 +1345,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1361,28 +1361,26 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1412,7 +1410,7 @@
     <xf numFmtId="10" fontId="6" fillId="8" borderId="39" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="8" fillId="8" borderId="40" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1433,9 +1431,203 @@
     <cellStyle name="Normal 4" xfId="3" xr:uid="{970C258E-AAE1-4AD6-8E1A-24DB03BEBBD2}"/>
     <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="215">
+  <dxfs count="105">
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1450,7 +1642,201 @@
         <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
-        <color indexed="12"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
       </font>
     </dxf>
     <dxf>
@@ -1577,1398 +1963,6 @@
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
       </font>
     </dxf>
     <dxf>
@@ -19432,8 +18426,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="112">
-        <v>46121</v>
+      <c r="A1" s="110">
+        <v>46269</v>
       </c>
       <c r="B1" s="93" t="s">
         <v>0</v>
@@ -19444,13 +18438,13 @@
       <c r="D1" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="E1" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="114" t="s">
+      <c r="F1" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="115" t="s">
+      <c r="G1" s="113" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="7" t="s">
@@ -19471,13 +18465,13 @@
       <c r="A2" s="96">
         <v>1</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="106" t="s">
+      <c r="D2" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="16">
@@ -19486,7 +18480,7 @@
       <c r="F2" s="77">
         <v>128.30000000000001</v>
       </c>
-      <c r="G2" s="116">
+      <c r="G2" s="114">
         <v>0</v>
       </c>
       <c r="I2" s="20"/>
@@ -19502,13 +18496,13 @@
       <c r="A3" s="98">
         <v>2</v>
       </c>
-      <c r="B3" s="105" t="s">
+      <c r="B3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="106" t="s">
+      <c r="D3" s="15" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="16">
@@ -19517,7 +18511,7 @@
       <c r="F3" s="77">
         <v>90.5</v>
       </c>
-      <c r="G3" s="116">
+      <c r="G3" s="114">
         <v>0</v>
       </c>
       <c r="H3" s="8"/>
@@ -19531,13 +18525,13 @@
       <c r="A4" s="96">
         <v>3</v>
       </c>
-      <c r="B4" s="105" t="s">
+      <c r="B4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="106" t="s">
+      <c r="D4" s="15" t="s">
         <v>13</v>
       </c>
       <c r="E4" s="16">
@@ -19546,7 +18540,7 @@
       <c r="F4" s="77">
         <v>44.805</v>
       </c>
-      <c r="G4" s="116">
+      <c r="G4" s="114">
         <v>0</v>
       </c>
       <c r="H4" s="8"/>
@@ -19560,13 +18554,13 @@
       <c r="A5" s="98">
         <v>4</v>
       </c>
-      <c r="B5" s="105" t="s">
+      <c r="B5" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="105" t="s">
+      <c r="C5" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="106" t="s">
+      <c r="D5" s="15" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="16">
@@ -19575,7 +18569,7 @@
       <c r="F5" s="77">
         <v>12.65</v>
       </c>
-      <c r="G5" s="116">
+      <c r="G5" s="114">
         <v>0</v>
       </c>
       <c r="H5" s="8"/>
@@ -19589,13 +18583,13 @@
       <c r="A6" s="96">
         <v>5</v>
       </c>
-      <c r="B6" s="105" t="s">
+      <c r="B6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="105" t="s">
+      <c r="C6" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="106" t="s">
+      <c r="D6" s="15" t="s">
         <v>17</v>
       </c>
       <c r="E6" s="16">
@@ -19604,7 +18598,7 @@
       <c r="F6" s="77">
         <v>216.2</v>
       </c>
-      <c r="G6" s="116">
+      <c r="G6" s="114">
         <v>0</v>
       </c>
       <c r="H6" s="8"/>
@@ -19618,13 +18612,13 @@
       <c r="A7" s="98">
         <v>6</v>
       </c>
-      <c r="B7" s="105" t="s">
+      <c r="B7" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="105" t="s">
+      <c r="C7" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="106" t="s">
+      <c r="D7" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="16">
@@ -19633,7 +18627,7 @@
       <c r="F7" s="77">
         <v>19.82</v>
       </c>
-      <c r="G7" s="116">
+      <c r="G7" s="114">
         <v>0</v>
       </c>
       <c r="H7" s="8"/>
@@ -19647,13 +18641,13 @@
       <c r="A8" s="96">
         <v>7</v>
       </c>
-      <c r="B8" s="105" t="s">
+      <c r="B8" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="105" t="s">
+      <c r="C8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="106" t="s">
+      <c r="D8" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E8" s="16">
@@ -19662,7 +18656,7 @@
       <c r="F8" s="77">
         <v>0.96</v>
       </c>
-      <c r="G8" s="116">
+      <c r="G8" s="114">
         <v>0</v>
       </c>
       <c r="H8" s="8"/>
@@ -19676,13 +18670,13 @@
       <c r="A9" s="98">
         <v>8</v>
       </c>
-      <c r="B9" s="105" t="s">
+      <c r="B9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="105" t="s">
+      <c r="C9" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="106" t="s">
+      <c r="D9" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="16">
@@ -19691,7 +18685,7 @@
       <c r="F9" s="77">
         <v>9.2100000000000009</v>
       </c>
-      <c r="G9" s="116">
+      <c r="G9" s="114">
         <v>0</v>
       </c>
       <c r="H9" s="8"/>
@@ -19705,13 +18699,13 @@
       <c r="A10" s="96">
         <v>9</v>
       </c>
-      <c r="B10" s="105" t="s">
+      <c r="B10" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="105" t="s">
+      <c r="C10" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="106" t="s">
+      <c r="D10" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="16">
@@ -19720,7 +18714,7 @@
       <c r="F10" s="77">
         <v>16.405000000000001</v>
       </c>
-      <c r="G10" s="116">
+      <c r="G10" s="114">
         <v>0</v>
       </c>
       <c r="H10" s="8"/>
@@ -19734,13 +18728,13 @@
       <c r="A11" s="98">
         <v>10</v>
       </c>
-      <c r="B11" s="105" t="s">
+      <c r="B11" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="105" t="s">
+      <c r="C11" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="106" t="s">
+      <c r="D11" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E11" s="16">
@@ -19749,7 +18743,7 @@
       <c r="F11" s="77">
         <v>18.64</v>
       </c>
-      <c r="G11" s="116">
+      <c r="G11" s="114">
         <v>0</v>
       </c>
       <c r="H11" s="8"/>
@@ -19764,8 +18758,8 @@
       <c r="B12" s="100"/>
       <c r="C12" s="101"/>
       <c r="D12" s="102"/>
-      <c r="E12" s="117"/>
-      <c r="F12" s="118" t="s">
+      <c r="E12" s="115"/>
+      <c r="F12" s="116" t="s">
         <v>28</v>
       </c>
       <c r="G12" s="39">
@@ -19825,13 +18819,13 @@
       <c r="A16" s="96">
         <v>1</v>
       </c>
-      <c r="B16" s="105" t="s">
+      <c r="B16" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="105" t="s">
+      <c r="C16" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="106" t="s">
+      <c r="D16" s="15" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="36">
@@ -19850,13 +18844,13 @@
       <c r="A17" s="98">
         <v>2</v>
       </c>
-      <c r="B17" s="105" t="s">
+      <c r="B17" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="105" t="s">
+      <c r="C17" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D17" s="106" t="s">
+      <c r="D17" s="15" t="s">
         <v>36</v>
       </c>
       <c r="E17" s="36">
@@ -19875,13 +18869,13 @@
       <c r="A18" s="96">
         <v>3</v>
       </c>
-      <c r="B18" s="105" t="s">
+      <c r="B18" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="105" t="s">
+      <c r="C18" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="106" t="s">
+      <c r="D18" s="15" t="s">
         <v>38</v>
       </c>
       <c r="E18" s="36">
@@ -19900,13 +18894,13 @@
       <c r="A19" s="98">
         <v>4</v>
       </c>
-      <c r="B19" s="105" t="s">
+      <c r="B19" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="105" t="s">
+      <c r="C19" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="106" t="s">
+      <c r="D19" s="15" t="s">
         <v>40</v>
       </c>
       <c r="E19" s="36">
@@ -19925,13 +18919,13 @@
       <c r="A20" s="96">
         <v>5</v>
       </c>
-      <c r="B20" s="105" t="s">
+      <c r="B20" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="105" t="s">
+      <c r="C20" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="106" t="s">
+      <c r="D20" s="15" t="s">
         <v>42</v>
       </c>
       <c r="E20" s="36">
@@ -19950,13 +18944,13 @@
       <c r="A21" s="98">
         <v>6</v>
       </c>
-      <c r="B21" s="105" t="s">
+      <c r="B21" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="105" t="s">
+      <c r="C21" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="106" t="s">
+      <c r="D21" s="15" t="s">
         <v>44</v>
       </c>
       <c r="E21" s="36">
@@ -19975,13 +18969,13 @@
       <c r="A22" s="96">
         <v>7</v>
       </c>
-      <c r="B22" s="105" t="s">
+      <c r="B22" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="105" t="s">
+      <c r="C22" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="106" t="s">
+      <c r="D22" s="15" t="s">
         <v>46</v>
       </c>
       <c r="E22" s="36">
@@ -20000,13 +18994,13 @@
       <c r="A23" s="98">
         <v>8</v>
       </c>
-      <c r="B23" s="105" t="s">
+      <c r="B23" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="105" t="s">
+      <c r="C23" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="106" t="s">
+      <c r="D23" s="15" t="s">
         <v>48</v>
       </c>
       <c r="E23" s="36">
@@ -20025,13 +19019,13 @@
       <c r="A24" s="96">
         <v>9</v>
       </c>
-      <c r="B24" s="105" t="s">
+      <c r="B24" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="105" t="s">
+      <c r="C24" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D24" s="106" t="s">
+      <c r="D24" s="15" t="s">
         <v>50</v>
       </c>
       <c r="E24" s="36">
@@ -20050,13 +19044,13 @@
       <c r="A25" s="98">
         <v>10</v>
       </c>
-      <c r="B25" s="105" t="s">
+      <c r="B25" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="105" t="s">
+      <c r="C25" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="106" t="s">
+      <c r="D25" s="15" t="s">
         <v>52</v>
       </c>
       <c r="E25" s="36">
@@ -20073,9 +19067,9 @@
     </row>
     <row r="26" spans="1:11" ht="15.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="96"/>
-      <c r="B26" s="105"/>
+      <c r="B26" s="14"/>
       <c r="C26" s="76"/>
-      <c r="D26" s="107"/>
+      <c r="D26" s="105"/>
       <c r="E26" s="36"/>
       <c r="F26" s="38" t="s">
         <v>28</v>
@@ -20097,11 +19091,11 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A27" s="108"/>
-      <c r="B27" s="109"/>
+      <c r="A27" s="106"/>
+      <c r="B27" s="107"/>
       <c r="C27" s="100"/>
-      <c r="D27" s="110"/>
-      <c r="E27" s="111"/>
+      <c r="D27" s="108"/>
+      <c r="E27" s="109"/>
       <c r="F27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27"/>
@@ -20123,13 +19117,13 @@
       <c r="D29" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="E29" s="113" t="s">
+      <c r="E29" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="F29" s="114" t="s">
+      <c r="F29" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="G29" s="115" t="s">
+      <c r="G29" s="113" t="s">
         <v>5</v>
       </c>
       <c r="H29" s="7" t="s">
@@ -20141,13 +19135,13 @@
       <c r="A30" s="96">
         <v>1</v>
       </c>
-      <c r="B30" s="105" t="s">
+      <c r="B30" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="105" t="s">
+      <c r="C30" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D30" s="106" t="s">
+      <c r="D30" s="15" t="s">
         <v>56</v>
       </c>
       <c r="E30" s="16">
@@ -20156,7 +19150,7 @@
       <c r="F30" s="77">
         <v>3.95</v>
       </c>
-      <c r="G30" s="116">
+      <c r="G30" s="114">
         <v>0</v>
       </c>
       <c r="H30"/>
@@ -20166,13 +19160,13 @@
       <c r="A31" s="98">
         <v>2</v>
       </c>
-      <c r="B31" s="105" t="s">
+      <c r="B31" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="C31" s="105" t="s">
+      <c r="C31" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="106" t="s">
+      <c r="D31" s="15" t="s">
         <v>58</v>
       </c>
       <c r="E31" s="16">
@@ -20181,7 +19175,7 @@
       <c r="F31" s="77">
         <v>28.76</v>
       </c>
-      <c r="G31" s="116">
+      <c r="G31" s="114">
         <v>0</v>
       </c>
       <c r="H31"/>
@@ -20191,13 +19185,13 @@
       <c r="A32" s="96">
         <v>3</v>
       </c>
-      <c r="B32" s="105" t="s">
+      <c r="B32" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C32" s="105" t="s">
+      <c r="C32" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="106" t="s">
+      <c r="D32" s="15" t="s">
         <v>60</v>
       </c>
       <c r="E32" s="16">
@@ -20206,7 +19200,7 @@
       <c r="F32" s="77">
         <v>0.28799999999999998</v>
       </c>
-      <c r="G32" s="116">
+      <c r="G32" s="114">
         <v>0</v>
       </c>
       <c r="H32"/>
@@ -20216,13 +19210,13 @@
       <c r="A33" s="98">
         <v>4</v>
       </c>
-      <c r="B33" s="105" t="s">
+      <c r="B33" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="105" t="s">
+      <c r="C33" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D33" s="106" t="s">
+      <c r="D33" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E33" s="16">
@@ -20231,7 +19225,7 @@
       <c r="F33" s="77">
         <v>19.600000000000001</v>
       </c>
-      <c r="G33" s="116">
+      <c r="G33" s="114">
         <v>0</v>
       </c>
       <c r="H33"/>
@@ -20241,13 +19235,13 @@
       <c r="A34" s="96">
         <v>5</v>
       </c>
-      <c r="B34" s="105" t="s">
+      <c r="B34" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="105" t="s">
+      <c r="C34" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="106" t="s">
+      <c r="D34" s="15" t="s">
         <v>65</v>
       </c>
       <c r="E34" s="16">
@@ -20256,7 +19250,7 @@
       <c r="F34" s="77">
         <v>1.095</v>
       </c>
-      <c r="G34" s="116">
+      <c r="G34" s="114">
         <v>0</v>
       </c>
       <c r="H34"/>
@@ -20266,13 +19260,13 @@
       <c r="A35" s="98">
         <v>6</v>
       </c>
-      <c r="B35" s="105" t="s">
+      <c r="B35" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="105" t="s">
+      <c r="C35" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D35" s="106" t="s">
+      <c r="D35" s="15" t="s">
         <v>67</v>
       </c>
       <c r="E35" s="16">
@@ -20281,7 +19275,7 @@
       <c r="F35" s="77">
         <v>4.92</v>
       </c>
-      <c r="G35" s="116">
+      <c r="G35" s="114">
         <v>0</v>
       </c>
       <c r="H35"/>
@@ -20291,13 +19285,13 @@
       <c r="A36" s="96">
         <v>7</v>
       </c>
-      <c r="B36" s="105" t="s">
+      <c r="B36" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="105" t="s">
+      <c r="C36" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D36" s="106" t="s">
+      <c r="D36" s="15" t="s">
         <v>69</v>
       </c>
       <c r="E36" s="16">
@@ -20306,7 +19300,7 @@
       <c r="F36" s="77">
         <v>32.5</v>
       </c>
-      <c r="G36" s="116">
+      <c r="G36" s="114">
         <v>0</v>
       </c>
       <c r="H36"/>
@@ -20316,13 +19310,13 @@
       <c r="A37" s="98">
         <v>8</v>
       </c>
-      <c r="B37" s="105" t="s">
+      <c r="B37" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="105" t="s">
+      <c r="C37" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="106" t="s">
+      <c r="D37" s="15" t="s">
         <v>71</v>
       </c>
       <c r="E37" s="16">
@@ -20331,7 +19325,7 @@
       <c r="F37" s="77">
         <v>0.46600000000000003</v>
       </c>
-      <c r="G37" s="116">
+      <c r="G37" s="114">
         <v>0</v>
       </c>
       <c r="H37"/>
@@ -20342,13 +19336,13 @@
       <c r="A38" s="96">
         <v>9</v>
       </c>
-      <c r="B38" s="105" t="s">
+      <c r="B38" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="105" t="s">
+      <c r="C38" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D38" s="106" t="s">
+      <c r="D38" s="15" t="s">
         <v>73</v>
       </c>
       <c r="E38" s="16">
@@ -20357,7 +19351,7 @@
       <c r="F38" s="77">
         <v>117.5</v>
       </c>
-      <c r="G38" s="116">
+      <c r="G38" s="114">
         <v>0</v>
       </c>
       <c r="H38"/>
@@ -20368,13 +19362,13 @@
       <c r="A39" s="98">
         <v>10</v>
       </c>
-      <c r="B39" s="105" t="s">
+      <c r="B39" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C39" s="105" t="s">
+      <c r="C39" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D39" s="106" t="s">
+      <c r="D39" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E39" s="16">
@@ -20383,22 +19377,22 @@
       <c r="F39" s="77">
         <v>5.14</v>
       </c>
-      <c r="G39" s="116">
+      <c r="G39" s="114">
         <v>0</v>
       </c>
       <c r="H39"/>
       <c r="I39"/>
     </row>
     <row r="40" spans="1:16" ht="16.3" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="125"/>
-      <c r="B40" s="126"/>
-      <c r="C40" s="127"/>
-      <c r="D40" s="128"/>
-      <c r="E40" s="129"/>
-      <c r="F40" s="118" t="s">
+      <c r="A40" s="123"/>
+      <c r="B40" s="124"/>
+      <c r="C40" s="125"/>
+      <c r="D40" s="126"/>
+      <c r="E40" s="127"/>
+      <c r="F40" s="116" t="s">
         <v>28</v>
       </c>
-      <c r="G40" s="130">
+      <c r="G40" s="128">
         <v>0</v>
       </c>
       <c r="H40" s="31" t="s">
@@ -20437,13 +19431,13 @@
       <c r="D42" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="E42" s="113" t="s">
+      <c r="E42" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="F42" s="114" t="s">
+      <c r="F42" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="G42" s="121" t="s">
+      <c r="G42" s="119" t="s">
         <v>5</v>
       </c>
       <c r="H42" s="7" t="s">
@@ -20455,12 +19449,12 @@
       <c r="A43" s="96">
         <v>1</v>
       </c>
-      <c r="B43" s="105"/>
-      <c r="C43" s="105"/>
-      <c r="D43" s="106"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="15"/>
       <c r="E43" s="16"/>
       <c r="F43" s="77"/>
-      <c r="G43" s="122" t="e">
+      <c r="G43" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H43"/>
@@ -20470,12 +19464,12 @@
       <c r="A44" s="98">
         <v>2</v>
       </c>
-      <c r="B44" s="105"/>
-      <c r="C44" s="105"/>
-      <c r="D44" s="106"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="15"/>
       <c r="E44" s="16"/>
       <c r="F44" s="77"/>
-      <c r="G44" s="122" t="e">
+      <c r="G44" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H44"/>
@@ -20485,12 +19479,12 @@
       <c r="A45" s="96">
         <v>3</v>
       </c>
-      <c r="B45" s="105"/>
-      <c r="C45" s="105"/>
-      <c r="D45" s="106"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="15"/>
       <c r="E45" s="16"/>
       <c r="F45" s="77"/>
-      <c r="G45" s="122" t="e">
+      <c r="G45" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H45"/>
@@ -20500,12 +19494,12 @@
       <c r="A46" s="98">
         <v>4</v>
       </c>
-      <c r="B46" s="105"/>
-      <c r="C46" s="105"/>
-      <c r="D46" s="106"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="15"/>
       <c r="E46" s="16"/>
       <c r="F46" s="77"/>
-      <c r="G46" s="122" t="e">
+      <c r="G46" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H46"/>
@@ -20515,12 +19509,12 @@
       <c r="A47" s="96">
         <v>5</v>
       </c>
-      <c r="B47" s="105"/>
-      <c r="C47" s="105"/>
-      <c r="D47" s="106"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="15"/>
       <c r="E47" s="16"/>
       <c r="F47" s="77"/>
-      <c r="G47" s="122" t="e">
+      <c r="G47" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H47"/>
@@ -20530,12 +19524,12 @@
       <c r="A48" s="98">
         <v>6</v>
       </c>
-      <c r="B48" s="105"/>
-      <c r="C48" s="105"/>
-      <c r="D48" s="106"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="15"/>
       <c r="E48" s="16"/>
       <c r="F48" s="77"/>
-      <c r="G48" s="122" t="e">
+      <c r="G48" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H48"/>
@@ -20545,12 +19539,12 @@
       <c r="A49" s="96">
         <v>7</v>
       </c>
-      <c r="B49" s="105"/>
-      <c r="C49" s="105"/>
-      <c r="D49" s="106"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="15"/>
       <c r="E49" s="16"/>
       <c r="F49" s="77"/>
-      <c r="G49" s="122" t="e">
+      <c r="G49" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H49"/>
@@ -20560,12 +19554,12 @@
       <c r="A50" s="98">
         <v>8</v>
       </c>
-      <c r="B50" s="105"/>
-      <c r="C50" s="105"/>
-      <c r="D50" s="106"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="15"/>
       <c r="E50" s="16"/>
       <c r="F50" s="77"/>
-      <c r="G50" s="122" t="e">
+      <c r="G50" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H50"/>
@@ -20575,12 +19569,12 @@
       <c r="A51" s="96">
         <v>9</v>
       </c>
-      <c r="B51" s="105"/>
-      <c r="C51" s="105"/>
-      <c r="D51" s="106"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="15"/>
       <c r="E51" s="16"/>
       <c r="F51" s="77"/>
-      <c r="G51" s="122" t="e">
+      <c r="G51" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H51"/>
@@ -20590,12 +19584,12 @@
       <c r="A52" s="98">
         <v>10</v>
       </c>
-      <c r="B52" s="105"/>
-      <c r="C52" s="105"/>
-      <c r="D52" s="106"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="15"/>
       <c r="E52" s="16"/>
       <c r="F52" s="77"/>
-      <c r="G52" s="122" t="e">
+      <c r="G52" s="120" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H52"/>
@@ -20606,11 +19600,11 @@
       <c r="B53" s="100"/>
       <c r="C53" s="101"/>
       <c r="D53" s="102"/>
-      <c r="E53" s="123"/>
-      <c r="F53" s="120" t="s">
+      <c r="E53" s="121"/>
+      <c r="F53" s="118" t="s">
         <v>28</v>
       </c>
-      <c r="G53" s="124" t="e">
+      <c r="G53" s="122" t="e">
         <v>#VALUE!</v>
       </c>
       <c r="H53" s="31" t="s">
@@ -20668,9 +19662,7 @@
       <c r="B56" s="75"/>
       <c r="C56" s="76"/>
       <c r="D56" s="75"/>
-      <c r="E56" s="97">
-        <v>16.405000000000001</v>
-      </c>
+      <c r="E56" s="97"/>
       <c r="F56" s="17"/>
       <c r="G56" s="53" t="e">
         <v>#VALUE!</v>
@@ -20684,9 +19676,7 @@
       <c r="B57" s="80"/>
       <c r="C57" s="26"/>
       <c r="D57" s="80"/>
-      <c r="E57" s="97">
-        <v>9.9320000000000004</v>
-      </c>
+      <c r="E57" s="97"/>
       <c r="F57" s="17"/>
       <c r="G57" s="53" t="e">
         <v>#VALUE!</v>
@@ -20701,9 +19691,7 @@
       <c r="B58" s="75"/>
       <c r="C58" s="76"/>
       <c r="D58" s="75"/>
-      <c r="E58" s="97">
-        <v>21.15</v>
-      </c>
+      <c r="E58" s="97"/>
       <c r="F58" s="17"/>
       <c r="G58" s="53" t="e">
         <v>#VALUE!</v>
@@ -20719,9 +19707,7 @@
       <c r="B59" s="80"/>
       <c r="C59" s="26"/>
       <c r="D59" s="80"/>
-      <c r="E59" s="97">
-        <v>35.159999999999997</v>
-      </c>
+      <c r="E59" s="97"/>
       <c r="F59" s="17"/>
       <c r="G59" s="53" t="e">
         <v>#VALUE!</v>
@@ -20737,9 +19723,7 @@
       <c r="B60" s="75"/>
       <c r="C60" s="76"/>
       <c r="D60" s="75"/>
-      <c r="E60" s="97">
-        <v>2.56</v>
-      </c>
+      <c r="E60" s="97"/>
       <c r="F60" s="17"/>
       <c r="G60" s="53" t="e">
         <v>#VALUE!</v>
@@ -20755,9 +19739,7 @@
       <c r="B61" s="80"/>
       <c r="C61" s="26"/>
       <c r="D61" s="80"/>
-      <c r="E61" s="97">
-        <v>30.45</v>
-      </c>
+      <c r="E61" s="97"/>
       <c r="F61" s="17"/>
       <c r="G61" s="53" t="e">
         <v>#VALUE!</v>
@@ -20773,9 +19755,7 @@
       <c r="B62" s="75"/>
       <c r="C62" s="76"/>
       <c r="D62" s="75"/>
-      <c r="E62" s="97">
-        <v>15.71</v>
-      </c>
+      <c r="E62" s="97"/>
       <c r="F62" s="17"/>
       <c r="G62" s="53" t="e">
         <v>#VALUE!</v>
@@ -20790,9 +19770,7 @@
       <c r="B63" s="80"/>
       <c r="C63" s="26"/>
       <c r="D63" s="80"/>
-      <c r="E63" s="97">
-        <v>46.9</v>
-      </c>
+      <c r="E63" s="97"/>
       <c r="F63" s="17"/>
       <c r="G63" s="53" t="e">
         <v>#VALUE!</v>
@@ -21231,7 +20209,7 @@
         <v>4</v>
       </c>
       <c r="B85" s="80"/>
-      <c r="C85" s="119"/>
+      <c r="C85" s="117"/>
       <c r="D85" s="80"/>
       <c r="E85" s="16"/>
       <c r="F85" s="77"/>
@@ -21246,7 +20224,7 @@
         <v>5</v>
       </c>
       <c r="B86" s="75"/>
-      <c r="C86" s="119"/>
+      <c r="C86" s="117"/>
       <c r="D86" s="75"/>
       <c r="E86" s="16"/>
       <c r="F86" s="77"/>
@@ -21261,7 +20239,7 @@
         <v>6</v>
       </c>
       <c r="B87" s="80"/>
-      <c r="C87" s="119"/>
+      <c r="C87" s="117"/>
       <c r="D87" s="80"/>
       <c r="E87" s="16"/>
       <c r="F87" s="77"/>
@@ -21291,7 +20269,7 @@
         <v>8</v>
       </c>
       <c r="B89" s="80"/>
-      <c r="C89" s="119"/>
+      <c r="C89" s="117"/>
       <c r="D89" s="80"/>
       <c r="E89" s="16"/>
       <c r="F89" s="77"/>
@@ -21337,7 +20315,7 @@
       <c r="C92" s="83"/>
       <c r="D92" s="54"/>
       <c r="E92" s="84"/>
-      <c r="F92" s="120" t="s">
+      <c r="F92" s="118" t="s">
         <v>28</v>
       </c>
       <c r="G92" s="50" t="e">
@@ -23788,434 +22766,428 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B56:B65">
-    <cfRule type="expression" dxfId="106" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="104" priority="6" stopIfTrue="1">
       <formula>IF(AO56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:B78">
-    <cfRule type="expression" dxfId="105" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="103" priority="4" stopIfTrue="1">
       <formula>IF(AO69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B81">
-    <cfRule type="expression" dxfId="104" priority="51" stopIfTrue="1">
+    <cfRule type="expression" dxfId="102" priority="51" stopIfTrue="1">
       <formula>IF(AN62&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B82:B91">
-    <cfRule type="expression" dxfId="103" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="101" priority="10" stopIfTrue="1">
       <formula>IF(AL82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="expression" dxfId="102" priority="47" stopIfTrue="1">
+    <cfRule type="expression" dxfId="100" priority="47" stopIfTrue="1">
       <formula>IF(AL91&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="expression" dxfId="101" priority="50" stopIfTrue="1">
+    <cfRule type="expression" dxfId="99" priority="50" stopIfTrue="1">
       <formula>IF(AN75&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:B105">
-    <cfRule type="expression" dxfId="100" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="98" priority="8" stopIfTrue="1">
       <formula>IF(AO96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B106">
-    <cfRule type="expression" dxfId="99" priority="48" stopIfTrue="1">
+    <cfRule type="expression" dxfId="97" priority="48" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="expression" dxfId="98" priority="49" stopIfTrue="1">
+    <cfRule type="expression" dxfId="96" priority="49" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D56:D65">
-    <cfRule type="expression" dxfId="97" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="95" priority="5" stopIfTrue="1">
       <formula>IF(AQ56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:D78">
-    <cfRule type="expression" dxfId="96" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="94" priority="3" stopIfTrue="1">
       <formula>IF(AQ69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82:D91">
-    <cfRule type="expression" dxfId="95" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="93" priority="9" stopIfTrue="1">
       <formula>IF(AN82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D96:D105">
-    <cfRule type="expression" dxfId="94" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="92" priority="7" stopIfTrue="1">
       <formula>IF(AQ96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" dxfId="93" priority="20" stopIfTrue="1">
+    <cfRule type="expression" dxfId="91" priority="20" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="92" priority="21" stopIfTrue="1">
+    <cfRule type="expression" dxfId="90" priority="21" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="91" priority="22" stopIfTrue="1">
+    <cfRule type="expression" dxfId="89" priority="22" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="90" priority="23" stopIfTrue="1">
+    <cfRule type="expression" dxfId="88" priority="23" stopIfTrue="1">
       <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="89" priority="24" stopIfTrue="1">
+    <cfRule type="expression" dxfId="87" priority="24" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="88" priority="25" stopIfTrue="1">
+    <cfRule type="expression" dxfId="86" priority="25" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" dxfId="87" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="85" priority="82" stopIfTrue="1">
+      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="84" priority="81" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="86" priority="82" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="85" priority="83" stopIfTrue="1">
+    <cfRule type="expression" dxfId="83" priority="83" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="84" priority="84" stopIfTrue="1">
-      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="83" priority="85" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="82" priority="86" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="81" priority="85" stopIfTrue="1">
+      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="80" priority="84" stopIfTrue="1">
+      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" dxfId="81" priority="87" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="80" priority="88" stopIfTrue="1">
+    <cfRule type="expression" dxfId="79" priority="91" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="79" priority="89" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="78" priority="90" stopIfTrue="1">
       <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="91" stopIfTrue="1">
+    <cfRule type="expression" dxfId="77" priority="89" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="76" priority="88" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="76" priority="92" stopIfTrue="1">
+    <cfRule type="expression" dxfId="75" priority="87" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="74" priority="92" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F56">
-    <cfRule type="expression" dxfId="75" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="73" priority="80" stopIfTrue="1">
+      <formula>IF($U254="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="72" priority="79" stopIfTrue="1">
+      <formula>IF($T254="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="71" priority="78" stopIfTrue="1">
+      <formula>IF($AN28="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F67">
+    <cfRule type="expression" dxfId="70" priority="77" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="78" stopIfTrue="1">
-      <formula>IF($AN28="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F57:F67">
+    <cfRule type="expression" dxfId="69" priority="94" stopIfTrue="1">
+      <formula>IF($AK29="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="79" stopIfTrue="1">
-      <formula>IF($T254="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="68" priority="95" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="80" stopIfTrue="1">
-      <formula>IF($U254="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="67" priority="96" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69">
+    <cfRule type="expression" dxfId="66" priority="98" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="97" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="64" priority="99" stopIfTrue="1">
+      <formula>IF($AJ43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="63" priority="100" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="62" priority="101" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" dxfId="71" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="61" priority="2" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F70:F78">
+    <cfRule type="expression" dxfId="60" priority="102" stopIfTrue="1">
+      <formula>IF($AJ42="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="59" priority="103" stopIfTrue="1">
+      <formula>IF($T267="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="58" priority="104" stopIfTrue="1">
+      <formula>IF($U267="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" dxfId="57" priority="105" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="56" priority="106" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="55" priority="107" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" dxfId="70" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="54" priority="66" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" dxfId="69" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="53" priority="67" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="52" priority="69" stopIfTrue="1">
+      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="51" priority="68" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="67" priority="69" stopIfTrue="1">
-      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" dxfId="66" priority="74" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="50" priority="76" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="75" stopIfTrue="1">
+    <cfRule type="expression" dxfId="49" priority="75" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="76" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="48" priority="74" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" dxfId="63" priority="70" stopIfTrue="1">
+    <cfRule type="expression" dxfId="47" priority="70" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" dxfId="62" priority="71" stopIfTrue="1">
+    <cfRule type="expression" dxfId="46" priority="73" stopIfTrue="1">
+      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="72" stopIfTrue="1">
+      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="71" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="61" priority="72" stopIfTrue="1">
-      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
+    <cfRule type="cellIs" dxfId="43" priority="54" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="73" stopIfTrue="1">
-      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    <cfRule type="cellIs" dxfId="42" priority="53" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="59" priority="53" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G28">
+    <cfRule type="cellIs" dxfId="41" priority="26" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="54" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:G41 G2:G12 G16:G26">
+    <cfRule type="cellIs" dxfId="40" priority="52" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G28 G2:G12">
-    <cfRule type="cellIs" dxfId="57" priority="26" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="56" priority="52" operator="greaterThan">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G54 G56:G67 G30:G41">
-    <cfRule type="cellIs" dxfId="55" priority="43" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G43:G54 G30:G41 G56:G67">
+    <cfRule type="cellIs" dxfId="39" priority="43" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" dxfId="54" priority="31" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="38" priority="34" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="33" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="32" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="32" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="33" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="35" priority="31" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="34" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" dxfId="50" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="34" priority="19" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="18" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="33" priority="18" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="19" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="32" priority="17" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" dxfId="47" priority="44" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="45" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="46" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="45" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="46" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="29" priority="44" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" dxfId="44" priority="27" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="30" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="29" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="28" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="28" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="29" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="27" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="30" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" dxfId="40" priority="39" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="41" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="40" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="39" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="42" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="41" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="42" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="21" priority="40" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" dxfId="36" priority="35" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="38" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="37" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="36" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="36" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="37" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="35" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="38" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H81">
+    <cfRule type="cellIs" dxfId="16" priority="16" operator="greaterThan">
+      <formula>$H81</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I12 I53 K53 I66 K66">
-    <cfRule type="cellIs" dxfId="32" priority="60" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="60" operator="greaterThan">
       <formula>$K12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26">
-    <cfRule type="cellIs" dxfId="31" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="11" operator="greaterThan">
       <formula>$K26</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I40 K40:K41">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="greaterThan">
+      <formula>$K40</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I75">
-    <cfRule type="cellIs" dxfId="30" priority="61" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="61" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I93:I94">
-    <cfRule type="cellIs" dxfId="29" priority="59" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="59" operator="greaterThan">
       <formula>$K93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I107">
-    <cfRule type="cellIs" dxfId="28" priority="58" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="58" operator="greaterThan">
       <formula>$K107</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I109">
-    <cfRule type="cellIs" dxfId="27" priority="56" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="56" operator="greaterThan">
       <formula>$K109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J97">
-    <cfRule type="cellIs" dxfId="26" priority="63" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="63" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J103">
-    <cfRule type="cellIs" dxfId="25" priority="62" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="62" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="cellIs" dxfId="24" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="14" operator="greaterThan">
       <formula>$K12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="cellIs" dxfId="23" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="13" operator="greaterThan">
       <formula>$K26</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K41">
-    <cfRule type="cellIs" dxfId="22" priority="12" operator="greaterThan">
-      <formula>$K41</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" dxfId="21" priority="16" operator="greaterThan">
-      <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="K93:K94">
-    <cfRule type="cellIs" dxfId="20" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="15" operator="greaterThan">
       <formula>$K93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K104">
-    <cfRule type="cellIs" dxfId="19" priority="64" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="64" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K107">
-    <cfRule type="cellIs" dxfId="18" priority="57" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="57" operator="greaterThan">
       <formula>$I107</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K109">
-    <cfRule type="cellIs" dxfId="17" priority="55" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="55" operator="greaterThan">
       <formula>$I109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P37:P38">
-    <cfRule type="cellIs" dxfId="16" priority="65" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="65" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F57:F67">
-    <cfRule type="expression" dxfId="15" priority="93" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="94" stopIfTrue="1">
-      <formula>IF($AK29="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="95" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="96" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69">
-    <cfRule type="expression" dxfId="11" priority="97" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="98" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="99" stopIfTrue="1">
-      <formula>IF($AJ43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="100" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="101" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F70:F78">
-    <cfRule type="expression" dxfId="6" priority="102" stopIfTrue="1">
-      <formula>IF($AJ42="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="103" stopIfTrue="1">
-      <formula>IF($T267="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="104" stopIfTrue="1">
-      <formula>IF($U267="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" dxfId="3" priority="105" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="106" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="107" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I40 K40">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
-      <formula>$K40</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>